<commit_message>
data: reasons for Stadtwerke Rostock, Traxys and Arcadian checked on their own documents; web: on-chain table names the demo claimant
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/web/downloads/netra-dataset.xlsx
+++ b/web/downloads/netra-dataset.xlsx
@@ -4361,7 +4361,7 @@
       <c r="O58" t="inlineStr"/>
       <c r="P58" t="inlineStr">
         <is>
-          <t>A small private company; no public emissions report was found.</t>
+          <t>Arcadian (trading as Hewitt) publishes product-level Climate Active disclosures for its lamb, pork and chicken, not a company total, so there is no company figure to show.</t>
         </is>
       </c>
       <c r="Q58" s="7" t="inlineStr"/>
@@ -5351,7 +5351,7 @@
       <c r="O74" t="inlineStr"/>
       <c r="P74" t="inlineStr">
         <is>
-          <t>No company emissions figure in tonnes was found in published reports.</t>
+          <t>The audited 2024 accounts mention the cost of CO2 allowances under the EU emissions trading scheme but give no emissions in tonnes, and the company website has no sustainability report. Plant-level EU ETS data has not been read yet.</t>
         </is>
       </c>
       <c r="Q74" s="7" t="n">
@@ -6391,7 +6391,7 @@
       <c r="O91" t="inlineStr"/>
       <c r="P91" t="inlineStr">
         <is>
-          <t>A commodity trader's South African carbon-tax offset account; Traxys publishes no emissions figure in tonnes that we could find.</t>
+          <t>Traxys's ESG page publishes policies and a conflict-minerals report, but no emissions figure in tonnes.</t>
         </is>
       </c>
       <c r="Q91" s="7" t="inlineStr"/>

</xml_diff>